<commit_message>
Version final de la tarea
</commit_message>
<xml_diff>
--- a/M4/m4t3_sesion3/Ejercicio_alumnos_clase3.xlsx
+++ b/M4/m4t3_sesion3/Ejercicio_alumnos_clase3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\derec\Desktop\Diplomado\ml-insurance-team-lab\M4\m4t3_sesion3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{747EE1ED-0A18-465E-AAB5-122033A2F368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCC5F9E-2FAD-4BB4-B338-98C6D9734735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{EBE4BF15-7C9B-437D-9962-39D9A1B5233E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="12" xr2:uid="{EBE4BF15-7C9B-437D-9962-39D9A1B5233E}"/>
   </bookViews>
   <sheets>
     <sheet name="Nombre Equipo" sheetId="3" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1792" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1807" uniqueCount="266">
   <si>
     <t>Calcula el IBNR del siguiente triangulo usando Chain Ladder, BF y Cape Cod</t>
   </si>
@@ -842,6 +842,51 @@
   <si>
     <t xml:space="preserve">~0.0412 años </t>
   </si>
+  <si>
+    <t>Chain Ladder para períodos antiguos debido a que ya se cuenta con la suficiente experiencia observada y BF/CC para los periodos recientes, ya que, utilizamos una estimación del loss ratio basada en la experiencia agregada de la cartera, esto reduce el sesgo por tener poca experiencia observada.</t>
+  </si>
+  <si>
+    <t>Sí, se utilizaron los últimos 8peridos, ya que presentan mayor estabilidad y son los más representativos respecto a la experiencia reciente.</t>
+  </si>
+  <si>
+    <t>Para el Triángulo 1, utilizando el patrón de pagos y la tasa de descuento considerada en el archivo, se obtiene una duración de Macaulay de aproximadamente 0.984 años, equivalente a alrededor de 11.8 meses. La duración modificada es aproximadamente 0.928 años</t>
+  </si>
+  <si>
+    <t>En 2019 también se usa Chain Ladder, pero aquí los pagos se estabilizan en niveles más bajos por ejemplo 1Q19 termina en 5.8M. En 2020 se aplica BF, porque los cálculos de CL incluso arrojan IBNR negativos en algunos trimestres, lo que indica que BF es más confiable. En 2021–2022 se recomienda Cape Cod, ya que ajusta el ELR endógeno y evita inconsistencias. En 2023–2024 se alterna CC y BF según maduración.</t>
+  </si>
+  <si>
+    <t>No se excluyeron periodos, se mantiene toda la información disponible para el desarrollo.</t>
+  </si>
+  <si>
+    <t>Para el Triángulo 2, la duración de Macaulay obtenida es aproximadamente 0.0412 años, con una duración modificada de aproximadamente 0.0388 años.</t>
+  </si>
+  <si>
+    <t>El backtesting resulta satisfactorio para el triángulo en los primeros trimestres (1Q19–4Q20). Las estimaciones obtenidas mediante Chain Ladder para los periodos maduros se mantienen prácticamente sin variaciones al incorporar información adicional. Asimismo, la estimación del loss ratio calculada con CC presenta cambios mínimos, lo que refuerza la elección de esta metodología para los trimestres comprendidos entre 1Q19 y 4Q20.</t>
+  </si>
+  <si>
+    <t>El backtesting resulta satisfactorio para el triángulo en los primeros trimestres (1Q19–4Q20). Las estimaciones obtenidas mediante Chain Ladder para los periodos maduros se mantienen prácticamente sin variaciones al incorporar información adicional. Asimismo, la estimación del loss ratio calculada con BF presenta cambios mínimos, lo que refuerza la elección de esta metodología para los trimestres comprendidos entre 1Q19 y 4Q20.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Alondra Abril Alarcón Alvarez </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Angelica Guadalupe Cravioto Perez</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Arturo Cortés Islas </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Dereck Favila Limón </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Ismael Ruiz Carbajal </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> José Julián Alcalá Alcántara </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Melissa González Cortés </t>
+  </si>
 </sst>
 </file>
 
@@ -862,7 +907,7 @@
     <numFmt numFmtId="173" formatCode="0.000"/>
     <numFmt numFmtId="174" formatCode="#,##0.0000000"/>
   </numFmts>
-  <fonts count="48" x14ac:knownFonts="1">
+  <fonts count="49" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1181,6 +1226,12 @@
       <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1614,7 +1665,7 @@
     <xf numFmtId="43" fontId="39" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="39" fillId="0" borderId="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="176">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1977,30 +2028,6 @@
     <xf numFmtId="2" fontId="35" fillId="12" borderId="19" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="9" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="19" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="18" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="8" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="6" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2046,6 +2073,30 @@
     <xf numFmtId="0" fontId="11" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="6" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="19" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="7" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="9" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="8" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2070,6 +2121,7 @@
     <xf numFmtId="0" fontId="33" fillId="8" borderId="21" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -2683,54 +2735,96 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F4823A5-D11A-4968-B386-9AD98FEBBAB4}">
-  <dimension ref="C3:C10"/>
+  <dimension ref="C3:D20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="3:3" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="3" spans="3:4" ht="18.75" x14ac:dyDescent="0.3">
       <c r="C3" s="8" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D4" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C5">
         <f>+C4+1</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D5" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">+C5+1</f>
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D6" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C7">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C9">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-    </row>
-    <row r="10" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
       <c r="C10">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
+      <c r="D10" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="14" spans="3:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="D14" s="175"/>
+    </row>
+    <row r="15" spans="3:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="D15" s="175"/>
+    </row>
+    <row r="16" spans="3:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="D16" s="175"/>
+    </row>
+    <row r="17" spans="4:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="D17" s="175"/>
+    </row>
+    <row r="18" spans="4:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="D18" s="175"/>
+    </row>
+    <row r="19" spans="4:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="D19" s="175"/>
+    </row>
+    <row r="20" spans="4:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="D20" s="175"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3658,15 +3752,15 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="161" t="s">
+      <c r="A32" s="153" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="161"/>
-      <c r="C32" s="161"/>
-      <c r="D32" s="161"/>
-      <c r="E32" s="161"/>
-      <c r="F32" s="161"/>
-      <c r="G32" s="161"/>
+      <c r="B32" s="153"/>
+      <c r="C32" s="153"/>
+      <c r="D32" s="153"/>
+      <c r="E32" s="153"/>
+      <c r="F32" s="153"/>
+      <c r="G32" s="153"/>
       <c r="H32" s="70">
         <f>SUM(H8:H31)</f>
         <v>-13281479.105080277</v>
@@ -3693,30 +3787,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="162" t="s">
+      <c r="A1" s="154" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="162"/>
-      <c r="C1" s="162"/>
-      <c r="D1" s="162"/>
-      <c r="E1" s="162"/>
-      <c r="F1" s="162"/>
-      <c r="G1" s="162"/>
-      <c r="H1" s="162"/>
-      <c r="I1" s="162"/>
+      <c r="B1" s="154"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="154"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="154"/>
+      <c r="I1" s="154"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="163" t="s">
+      <c r="A2" s="155" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="163"/>
-      <c r="C2" s="163"/>
-      <c r="D2" s="163"/>
-      <c r="E2" s="163"/>
-      <c r="F2" s="163"/>
-      <c r="G2" s="163"/>
-      <c r="H2" s="163"/>
-      <c r="I2" s="163"/>
+      <c r="B2" s="155"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="155"/>
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4673,14 +4767,14 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="164" t="s">
+      <c r="A32" s="156" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="165"/>
-      <c r="C32" s="165"/>
-      <c r="D32" s="165"/>
-      <c r="E32" s="165"/>
-      <c r="F32" s="166"/>
+      <c r="B32" s="157"/>
+      <c r="C32" s="157"/>
+      <c r="D32" s="157"/>
+      <c r="E32" s="157"/>
+      <c r="F32" s="158"/>
       <c r="G32" s="80">
         <f>SUM(G8:G31)</f>
         <v>437449617.16139412</v>
@@ -4720,28 +4814,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="146" t="s">
+      <c r="B1" s="163" t="s">
         <v>153</v>
       </c>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
+      <c r="C1" s="163"/>
+      <c r="D1" s="163"/>
+      <c r="E1" s="163"/>
+      <c r="F1" s="163"/>
+      <c r="G1" s="163"/>
+      <c r="H1" s="163"/>
+      <c r="I1" s="163"/>
     </row>
     <row r="2" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="147" t="s">
+      <c r="B2" s="164" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="147"/>
-      <c r="D2" s="147"/>
-      <c r="E2" s="147"/>
-      <c r="F2" s="147"/>
-      <c r="G2" s="147"/>
-      <c r="H2" s="147"/>
-      <c r="I2" s="147"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="164"/>
+      <c r="G2" s="164"/>
+      <c r="H2" s="164"/>
+      <c r="I2" s="164"/>
       <c r="N2" s="28" t="s">
         <v>245</v>
       </c>
@@ -4752,12 +4846,12 @@
       </c>
     </row>
     <row r="4" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="148" t="s">
+      <c r="B4" s="161" t="s">
         <v>155</v>
       </c>
-      <c r="C4" s="148"/>
-      <c r="D4" s="148"/>
-      <c r="E4" s="148"/>
+      <c r="C4" s="161"/>
+      <c r="D4" s="161"/>
+      <c r="E4" s="161"/>
       <c r="I4" s="28" t="s">
         <v>245</v>
       </c>
@@ -4770,14 +4864,14 @@
         <f>'2_CL'!AC33</f>
         <v>-12440003.44670379</v>
       </c>
-      <c r="D5" s="149" t="s">
+      <c r="D5" s="165" t="s">
         <v>157</v>
       </c>
-      <c r="E5" s="149"/>
-      <c r="F5" s="149"/>
-      <c r="G5" s="149"/>
-      <c r="H5" s="149"/>
-      <c r="I5" s="149"/>
+      <c r="E5" s="165"/>
+      <c r="F5" s="165"/>
+      <c r="G5" s="165"/>
+      <c r="H5" s="165"/>
+      <c r="I5" s="165"/>
     </row>
     <row r="6" spans="2:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="83" t="s">
@@ -4787,14 +4881,14 @@
         <f>IF(I4="Anual",Triangulo2!E5, POWER(1+Triangulo2!E5,0.25)-1)</f>
         <v>1.4673846168659299E-2</v>
       </c>
-      <c r="D6" s="149" t="s">
+      <c r="D6" s="165" t="s">
         <v>159</v>
       </c>
-      <c r="E6" s="149"/>
-      <c r="F6" s="149"/>
-      <c r="G6" s="149"/>
-      <c r="H6" s="149"/>
-      <c r="I6" s="149"/>
+      <c r="E6" s="165"/>
+      <c r="F6" s="165"/>
+      <c r="G6" s="165"/>
+      <c r="H6" s="165"/>
+      <c r="I6" s="165"/>
       <c r="J6" s="86">
         <v>0.04</v>
       </c>
@@ -4806,14 +4900,14 @@
       <c r="C7" s="85">
         <v>0.01</v>
       </c>
-      <c r="D7" s="149" t="s">
+      <c r="D7" s="165" t="s">
         <v>161</v>
       </c>
-      <c r="E7" s="149"/>
-      <c r="F7" s="149"/>
-      <c r="G7" s="149"/>
-      <c r="H7" s="149"/>
-      <c r="I7" s="149"/>
+      <c r="E7" s="165"/>
+      <c r="F7" s="165"/>
+      <c r="G7" s="165"/>
+      <c r="H7" s="165"/>
+      <c r="I7" s="165"/>
     </row>
     <row r="8" spans="2:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="83" t="s">
@@ -4822,26 +4916,26 @@
       <c r="C8" s="85">
         <v>0.4</v>
       </c>
-      <c r="D8" s="149" t="s">
+      <c r="D8" s="165" t="s">
         <v>163</v>
       </c>
-      <c r="E8" s="149"/>
-      <c r="F8" s="149"/>
-      <c r="G8" s="149"/>
-      <c r="H8" s="149"/>
-      <c r="I8" s="149"/>
+      <c r="E8" s="165"/>
+      <c r="F8" s="165"/>
+      <c r="G8" s="165"/>
+      <c r="H8" s="165"/>
+      <c r="I8" s="165"/>
     </row>
     <row r="10" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="148" t="s">
+      <c r="B10" s="161" t="s">
         <v>164</v>
       </c>
-      <c r="C10" s="148"/>
-      <c r="D10" s="148"/>
-      <c r="E10" s="148"/>
-      <c r="F10" s="148"/>
-      <c r="G10" s="148"/>
-      <c r="H10" s="148"/>
-      <c r="I10" s="148"/>
+      <c r="C10" s="161"/>
+      <c r="D10" s="161"/>
+      <c r="E10" s="161"/>
+      <c r="F10" s="161"/>
+      <c r="G10" s="161"/>
+      <c r="H10" s="161"/>
+      <c r="I10" s="161"/>
     </row>
     <row r="11" spans="2:14" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="87" t="s">
@@ -5827,16 +5921,16 @@
       </c>
     </row>
     <row r="38" spans="2:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="150" t="s">
+      <c r="B38" s="166" t="s">
         <v>173</v>
       </c>
-      <c r="C38" s="150"/>
-      <c r="D38" s="150"/>
-      <c r="E38" s="150"/>
-      <c r="F38" s="150"/>
-      <c r="G38" s="150"/>
-      <c r="H38" s="150"/>
-      <c r="I38" s="150"/>
+      <c r="C38" s="166"/>
+      <c r="D38" s="166"/>
+      <c r="E38" s="166"/>
+      <c r="F38" s="166"/>
+      <c r="G38" s="166"/>
+      <c r="H38" s="166"/>
+      <c r="I38" s="166"/>
     </row>
     <row r="39" spans="2:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="101" t="s">
@@ -5849,15 +5943,15 @@
       <c r="D39" s="103" t="s">
         <v>175</v>
       </c>
-      <c r="E39" s="144" t="s">
+      <c r="E39" s="162" t="s">
         <v>176</v>
       </c>
-      <c r="F39" s="144"/>
-      <c r="G39" s="144"/>
-      <c r="H39" s="145" t="s">
+      <c r="F39" s="162"/>
+      <c r="G39" s="162"/>
+      <c r="H39" s="160" t="s">
         <v>250</v>
       </c>
-      <c r="I39" s="145"/>
+      <c r="I39" s="160"/>
     </row>
     <row r="40" spans="2:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="2:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -5871,15 +5965,15 @@
       <c r="D41" s="103" t="s">
         <v>175</v>
       </c>
-      <c r="E41" s="144" t="s">
+      <c r="E41" s="162" t="s">
         <v>178</v>
       </c>
-      <c r="F41" s="144"/>
-      <c r="G41" s="144"/>
-      <c r="H41" s="145" t="s">
+      <c r="F41" s="162"/>
+      <c r="G41" s="162"/>
+      <c r="H41" s="160" t="s">
         <v>249</v>
       </c>
-      <c r="I41" s="145"/>
+      <c r="I41" s="160"/>
       <c r="J41" s="100">
         <f>+K36/(1+C6)</f>
         <v>4.0580076248649254E-2</v>
@@ -5895,28 +5989,28 @@
         <v>-0.54096134319812939</v>
       </c>
       <c r="D43" s="106"/>
-      <c r="E43" s="151" t="s">
+      <c r="E43" s="159" t="s">
         <v>180</v>
       </c>
-      <c r="F43" s="151"/>
-      <c r="G43" s="151"/>
-      <c r="H43" s="145" t="s">
+      <c r="F43" s="159"/>
+      <c r="G43" s="159"/>
+      <c r="H43" s="160" t="s">
         <v>181</v>
       </c>
-      <c r="I43" s="145"/>
+      <c r="I43" s="160"/>
     </row>
     <row r="44" spans="2:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="148" t="s">
+      <c r="B46" s="161" t="s">
         <v>182</v>
       </c>
-      <c r="C46" s="148"/>
-      <c r="D46" s="148"/>
-      <c r="E46" s="148"/>
-      <c r="F46" s="148"/>
-      <c r="G46" s="148"/>
-      <c r="H46" s="148"/>
-      <c r="I46" s="148"/>
+      <c r="C46" s="161"/>
+      <c r="D46" s="161"/>
+      <c r="E46" s="161"/>
+      <c r="F46" s="161"/>
+      <c r="G46" s="161"/>
+      <c r="H46" s="161"/>
+      <c r="I46" s="161"/>
     </row>
     <row r="47" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="107" t="s">
@@ -6062,24 +6156,24 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="B46:I46"/>
-    <mergeCell ref="E41:G41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="D6:I6"/>
     <mergeCell ref="D7:I7"/>
     <mergeCell ref="D8:I8"/>
     <mergeCell ref="B10:I10"/>
     <mergeCell ref="B38:I38"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="H39:I39"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="H41:I41"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4" xr:uid="{1C3F4381-2069-4F96-9919-02644A1609DF}">
       <formula1>$N$2:$N$3</formula1>
     </dataValidation>
@@ -6148,34 +6242,34 @@
       <c r="AA1" s="169"/>
     </row>
     <row r="3" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A3" s="148" t="s">
+      <c r="A3" s="161" t="s">
         <v>198</v>
       </c>
-      <c r="B3" s="148"/>
-      <c r="C3" s="148"/>
-      <c r="D3" s="148"/>
-      <c r="E3" s="148"/>
-      <c r="F3" s="148"/>
-      <c r="G3" s="148"/>
-      <c r="H3" s="148"/>
-      <c r="I3" s="148"/>
-      <c r="J3" s="148"/>
-      <c r="K3" s="148"/>
-      <c r="L3" s="148"/>
-      <c r="M3" s="148"/>
-      <c r="N3" s="148"/>
-      <c r="O3" s="148"/>
-      <c r="P3" s="148"/>
-      <c r="Q3" s="148"/>
-      <c r="R3" s="148"/>
-      <c r="S3" s="148"/>
-      <c r="T3" s="148"/>
-      <c r="U3" s="148"/>
-      <c r="V3" s="148"/>
-      <c r="W3" s="148"/>
-      <c r="X3" s="148"/>
-      <c r="Y3" s="148"/>
-      <c r="Z3" s="148"/>
+      <c r="B3" s="161"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="161"/>
+      <c r="K3" s="161"/>
+      <c r="L3" s="161"/>
+      <c r="M3" s="161"/>
+      <c r="N3" s="161"/>
+      <c r="O3" s="161"/>
+      <c r="P3" s="161"/>
+      <c r="Q3" s="161"/>
+      <c r="R3" s="161"/>
+      <c r="S3" s="161"/>
+      <c r="T3" s="161"/>
+      <c r="U3" s="161"/>
+      <c r="V3" s="161"/>
+      <c r="W3" s="161"/>
+      <c r="X3" s="161"/>
+      <c r="Y3" s="161"/>
+      <c r="Z3" s="161"/>
     </row>
     <row r="4" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="107" t="s">
@@ -10240,33 +10334,33 @@
       </c>
     </row>
     <row r="31" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A31" s="148" t="s">
+      <c r="A31" s="161" t="s">
         <v>207</v>
       </c>
-      <c r="B31" s="148"/>
-      <c r="C31" s="148"/>
-      <c r="D31" s="148"/>
-      <c r="E31" s="148"/>
-      <c r="F31" s="148"/>
-      <c r="G31" s="148"/>
-      <c r="H31" s="148"/>
-      <c r="I31" s="148"/>
-      <c r="J31" s="148"/>
-      <c r="K31" s="148"/>
-      <c r="L31" s="148"/>
-      <c r="M31" s="148"/>
-      <c r="N31" s="148"/>
-      <c r="O31" s="148"/>
-      <c r="P31" s="148"/>
-      <c r="Q31" s="148"/>
-      <c r="R31" s="148"/>
-      <c r="S31" s="148"/>
-      <c r="T31" s="148"/>
-      <c r="U31" s="148"/>
-      <c r="V31" s="148"/>
-      <c r="W31" s="148"/>
-      <c r="X31" s="148"/>
-      <c r="Y31" s="148"/>
+      <c r="B31" s="161"/>
+      <c r="C31" s="161"/>
+      <c r="D31" s="161"/>
+      <c r="E31" s="161"/>
+      <c r="F31" s="161"/>
+      <c r="G31" s="161"/>
+      <c r="H31" s="161"/>
+      <c r="I31" s="161"/>
+      <c r="J31" s="161"/>
+      <c r="K31" s="161"/>
+      <c r="L31" s="161"/>
+      <c r="M31" s="161"/>
+      <c r="N31" s="161"/>
+      <c r="O31" s="161"/>
+      <c r="P31" s="161"/>
+      <c r="Q31" s="161"/>
+      <c r="R31" s="161"/>
+      <c r="S31" s="161"/>
+      <c r="T31" s="161"/>
+      <c r="U31" s="161"/>
+      <c r="V31" s="161"/>
+      <c r="W31" s="161"/>
+      <c r="X31" s="161"/>
+      <c r="Y31" s="161"/>
     </row>
     <row r="32" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A32" s="107" t="s">
@@ -15375,50 +15469,62 @@
       <c r="D8" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="G8" t="s">
+        <v>251</v>
+      </c>
     </row>
     <row r="9" spans="3:27" x14ac:dyDescent="0.25">
       <c r="D9" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G9" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="10" spans="3:27" x14ac:dyDescent="0.25">
       <c r="D10" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="G10" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row r="11" spans="3:27" x14ac:dyDescent="0.25">
       <c r="D11" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="G11" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="13" spans="3:27" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="C13" s="152" t="s">
+      <c r="C13" s="144" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="152"/>
-      <c r="E13" s="152"/>
-      <c r="F13" s="152"/>
-      <c r="G13" s="152"/>
-      <c r="H13" s="152"/>
-      <c r="I13" s="152"/>
-      <c r="J13" s="152"/>
-      <c r="K13" s="152"/>
-      <c r="L13" s="152"/>
-      <c r="M13" s="152"/>
-      <c r="N13" s="152"/>
-      <c r="O13" s="152"/>
-      <c r="P13" s="152"/>
-      <c r="Q13" s="152"/>
-      <c r="R13" s="152"/>
-      <c r="S13" s="152"/>
-      <c r="T13" s="152"/>
-      <c r="U13" s="152"/>
-      <c r="V13" s="152"/>
-      <c r="W13" s="152"/>
-      <c r="X13" s="152"/>
-      <c r="Y13" s="152"/>
-      <c r="Z13" s="152"/>
-      <c r="AA13" s="152"/>
+      <c r="D13" s="144"/>
+      <c r="E13" s="144"/>
+      <c r="F13" s="144"/>
+      <c r="G13" s="144"/>
+      <c r="H13" s="144"/>
+      <c r="I13" s="144"/>
+      <c r="J13" s="144"/>
+      <c r="K13" s="144"/>
+      <c r="L13" s="144"/>
+      <c r="M13" s="144"/>
+      <c r="N13" s="144"/>
+      <c r="O13" s="144"/>
+      <c r="P13" s="144"/>
+      <c r="Q13" s="144"/>
+      <c r="R13" s="144"/>
+      <c r="S13" s="144"/>
+      <c r="T13" s="144"/>
+      <c r="U13" s="144"/>
+      <c r="V13" s="144"/>
+      <c r="W13" s="144"/>
+      <c r="X13" s="144"/>
+      <c r="Y13" s="144"/>
+      <c r="Z13" s="144"/>
+      <c r="AA13" s="144"/>
     </row>
     <row r="15" spans="3:27" x14ac:dyDescent="0.25">
       <c r="D15" s="10">
@@ -17392,33 +17498,33 @@
     <row r="41" spans="1:27" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A41" s="12"/>
       <c r="B41" s="12"/>
-      <c r="C41" s="152" t="s">
+      <c r="C41" s="144" t="s">
         <v>45</v>
       </c>
-      <c r="D41" s="152"/>
-      <c r="E41" s="152"/>
-      <c r="F41" s="152"/>
-      <c r="G41" s="152"/>
-      <c r="H41" s="152"/>
-      <c r="I41" s="152"/>
-      <c r="J41" s="152"/>
-      <c r="K41" s="152"/>
-      <c r="L41" s="152"/>
-      <c r="M41" s="152"/>
-      <c r="N41" s="152"/>
-      <c r="O41" s="152"/>
-      <c r="P41" s="152"/>
-      <c r="Q41" s="152"/>
-      <c r="R41" s="152"/>
-      <c r="S41" s="152"/>
-      <c r="T41" s="152"/>
-      <c r="U41" s="152"/>
-      <c r="V41" s="152"/>
-      <c r="W41" s="152"/>
-      <c r="X41" s="152"/>
-      <c r="Y41" s="152"/>
-      <c r="Z41" s="152"/>
-      <c r="AA41" s="152"/>
+      <c r="D41" s="144"/>
+      <c r="E41" s="144"/>
+      <c r="F41" s="144"/>
+      <c r="G41" s="144"/>
+      <c r="H41" s="144"/>
+      <c r="I41" s="144"/>
+      <c r="J41" s="144"/>
+      <c r="K41" s="144"/>
+      <c r="L41" s="144"/>
+      <c r="M41" s="144"/>
+      <c r="N41" s="144"/>
+      <c r="O41" s="144"/>
+      <c r="P41" s="144"/>
+      <c r="Q41" s="144"/>
+      <c r="R41" s="144"/>
+      <c r="S41" s="144"/>
+      <c r="T41" s="144"/>
+      <c r="U41" s="144"/>
+      <c r="V41" s="144"/>
+      <c r="W41" s="144"/>
+      <c r="X41" s="144"/>
+      <c r="Y41" s="144"/>
+      <c r="Z41" s="144"/>
+      <c r="AA41" s="144"/>
     </row>
     <row r="43" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D43" s="10">
@@ -19438,18 +19544,18 @@
       <c r="J76" s="1"/>
     </row>
     <row r="77" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="F77" s="153" t="s">
+      <c r="F77" s="145" t="s">
         <v>36</v>
       </c>
-      <c r="G77" s="153"/>
-      <c r="H77" s="153"/>
-      <c r="I77" s="153"/>
-      <c r="J77" s="154" t="s">
+      <c r="G77" s="145"/>
+      <c r="H77" s="145"/>
+      <c r="I77" s="145"/>
+      <c r="J77" s="146" t="s">
         <v>37</v>
       </c>
-      <c r="K77" s="154"/>
-      <c r="L77" s="154"/>
-      <c r="M77" s="154"/>
+      <c r="K77" s="146"/>
+      <c r="L77" s="146"/>
+      <c r="M77" s="146"/>
     </row>
     <row r="78" spans="2:27" x14ac:dyDescent="0.25">
       <c r="D78" s="4" t="s">
@@ -19509,7 +19615,10 @@
         <f>+'1_CC'!I8</f>
         <v>14725385</v>
       </c>
-      <c r="I79" s="1"/>
+      <c r="I79" s="1" t="str">
+        <f>IF(MAX(F79:H79)=F79,"Chain Ladder",IF(MAX(F79:H79)=G79,"BF","CC"))</f>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J79" s="1">
         <f>+'1_CL'!AC4</f>
         <v>0</v>
@@ -19521,6 +19630,10 @@
       <c r="L79" s="79">
         <f>+'1_CC'!H8</f>
         <v>0</v>
+      </c>
+      <c r="M79" s="1" t="str">
+        <f>IF(MAX(J79:L79)=J79,"Chain Ladder",IF(MAX(J79:L79)=K79,"BF","CC"))</f>
+        <v>Chain Ladder</v>
       </c>
     </row>
     <row r="80" spans="2:27" x14ac:dyDescent="0.25">
@@ -19550,7 +19663,10 @@
         <f>+'1_CC'!I9</f>
         <v>17735300.381189957</v>
       </c>
-      <c r="I80" s="1"/>
+      <c r="I80" s="1" t="str">
+        <f t="shared" ref="I80:I102" si="30">IF(MAX(F80:H80)=F80,"Chain Ladder",IF(MAX(F80:H80)=G80,"BF","CC"))</f>
+        <v>CC</v>
+      </c>
       <c r="J80" s="1">
         <f>+'1_CL'!AC5</f>
         <v>19.270448435097933</v>
@@ -19563,10 +19679,14 @@
         <f>+'1_CC'!H9</f>
         <v>21.381189957795133</v>
       </c>
-    </row>
-    <row r="81" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M80" s="1" t="str">
+        <f t="shared" ref="M80:M102" si="31">IF(MAX(J80:L80)=J80,"Chain Ladder",IF(MAX(J80:L80)=K80,"BF","CC"))</f>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="81" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B81">
-        <f t="shared" ref="B81:B102" si="30">+B80-1</f>
+        <f t="shared" ref="B81:B102" si="32">+B80-1</f>
         <v>22</v>
       </c>
       <c r="C81" s="7" t="s">
@@ -19591,7 +19711,10 @@
         <f>+'1_CC'!I10</f>
         <v>11881775.010277927</v>
       </c>
-      <c r="I81" s="1"/>
+      <c r="I81" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J81" s="1">
         <f>+'1_CL'!AC6</f>
         <v>19.864941546693444</v>
@@ -19604,10 +19727,14 @@
         <f>+'1_CC'!H10</f>
         <v>14.010277927212726</v>
       </c>
-    </row>
-    <row r="82" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M81" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="82" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B82">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>21</v>
       </c>
       <c r="C82" s="7" t="s">
@@ -19632,7 +19759,10 @@
         <f>+'1_CC'!I11</f>
         <v>19461723.624914289</v>
       </c>
-      <c r="I82" s="1"/>
+      <c r="I82" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J82" s="1">
         <f>+'1_CL'!AC7</f>
         <v>54.921350959688425</v>
@@ -19645,10 +19775,14 @@
         <f>+'1_CC'!H11</f>
         <v>73.624914289551938</v>
       </c>
-    </row>
-    <row r="83" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M82" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="83" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B83">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>20</v>
       </c>
       <c r="C83" s="7" t="s">
@@ -19673,7 +19807,10 @@
         <f>+'1_CC'!I12</f>
         <v>11816207.757040838</v>
       </c>
-      <c r="I83" s="1"/>
+      <c r="I83" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J83" s="1">
         <f>+'1_CL'!AC8</f>
         <v>69.088412698358297</v>
@@ -19686,10 +19823,14 @@
         <f>+'1_CC'!H12</f>
         <v>34.757040837522176</v>
       </c>
-    </row>
-    <row r="84" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M83" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="84" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B84">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>19</v>
       </c>
       <c r="C84" s="7" t="s">
@@ -19714,7 +19855,10 @@
         <f>+'1_CC'!I13</f>
         <v>13048641.692080954</v>
       </c>
-      <c r="I84" s="1"/>
+      <c r="I84" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J84" s="1">
         <f>+'1_CL'!AC9</f>
         <v>202.94963217712939</v>
@@ -19727,10 +19871,14 @@
         <f>+'1_CC'!H13</f>
         <v>170.69208095478891</v>
       </c>
-    </row>
-    <row r="85" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M84" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="85" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B85">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>18</v>
       </c>
       <c r="C85" s="7" t="s">
@@ -19755,7 +19903,10 @@
         <f>+'1_CC'!I14</f>
         <v>10840895.278688349</v>
       </c>
-      <c r="I85" s="1"/>
+      <c r="I85" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J85" s="1">
         <f>+'1_CL'!AC10</f>
         <v>522.1830773986876</v>
@@ -19768,10 +19919,14 @@
         <f>+'1_CC'!H14</f>
         <v>755.27868834827279</v>
       </c>
-    </row>
-    <row r="86" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M85" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="86" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B86">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>17</v>
       </c>
       <c r="C86" s="7" t="s">
@@ -19796,7 +19951,10 @@
         <f>+'1_CC'!I15</f>
         <v>14113128.649370886</v>
       </c>
-      <c r="I86" s="1"/>
+      <c r="I86" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J86" s="1">
         <f>+'1_CL'!AC11</f>
         <v>1652.4212332814932</v>
@@ -19809,10 +19967,14 @@
         <f>+'1_CC'!H15</f>
         <v>1992.6493708862381</v>
       </c>
-    </row>
-    <row r="87" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M86" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="87" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B87">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>16</v>
       </c>
       <c r="C87" s="7" t="s">
@@ -19837,7 +19999,10 @@
         <f>+'1_CC'!I16</f>
         <v>15732024.266389269</v>
       </c>
-      <c r="I87" s="1"/>
+      <c r="I87" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J87" s="1">
         <f>+'1_CL'!AC12</f>
         <v>4044.6840435676277</v>
@@ -19850,10 +20015,14 @@
         <f>+'1_CC'!H16</f>
         <v>2690.2663892691367</v>
       </c>
-    </row>
-    <row r="88" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M87" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="88" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B88">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>15</v>
       </c>
       <c r="C88" s="7" t="s">
@@ -19878,7 +20047,10 @@
         <f>+'1_CC'!I17</f>
         <v>14348952.519663077</v>
       </c>
-      <c r="I88" s="1"/>
+      <c r="I88" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J88" s="1">
         <f>+'1_CL'!AC13</f>
         <v>8101.782536027953</v>
@@ -19891,10 +20063,14 @@
         <f>+'1_CC'!H17</f>
         <v>5356.5196630770133</v>
       </c>
-    </row>
-    <row r="89" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M88" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="89" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B89">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>14</v>
       </c>
       <c r="C89" s="7" t="s">
@@ -19919,7 +20095,10 @@
         <f>+'1_CC'!I18</f>
         <v>15146435.277860068</v>
       </c>
-      <c r="I89" s="1"/>
+      <c r="I89" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J89" s="1">
         <f>+'1_CL'!AC14</f>
         <v>17451.426473489031</v>
@@ -19932,10 +20111,14 @@
         <f>+'1_CC'!H18</f>
         <v>26500.277860067999</v>
       </c>
-    </row>
-    <row r="90" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M89" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="90" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B90">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>13</v>
       </c>
       <c r="C90" s="7" t="s">
@@ -19960,7 +20143,10 @@
         <f>+'1_CC'!I19</f>
         <v>18774844.635980409</v>
       </c>
-      <c r="I90" s="1"/>
+      <c r="I90" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J90" s="1">
         <f>+'1_CL'!AC15</f>
         <v>42921.810095321387</v>
@@ -19973,10 +20159,14 @@
         <f>+'1_CC'!H19</f>
         <v>44820.635980407933</v>
       </c>
-    </row>
-    <row r="91" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M90" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="91" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B91">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>12</v>
       </c>
       <c r="C91" s="7" t="s">
@@ -20001,7 +20191,10 @@
         <f>+'1_CC'!I20</f>
         <v>19692980.654884461</v>
       </c>
-      <c r="I91" s="1"/>
+      <c r="I91" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J91" s="1">
         <f>+'1_CL'!AC16</f>
         <v>89289.649264484644</v>
@@ -20014,10 +20207,14 @@
         <f>+'1_CC'!H20</f>
         <v>65626.654884462769</v>
       </c>
-    </row>
-    <row r="92" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M91" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="92" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B92">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>11</v>
       </c>
       <c r="C92" s="7" t="s">
@@ -20042,7 +20239,10 @@
         <f>+'1_CC'!I21</f>
         <v>20265011.027012475</v>
       </c>
-      <c r="I92" s="1"/>
+      <c r="I92" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J92" s="1">
         <f>+'1_CL'!AC17</f>
         <v>168988.8463203311</v>
@@ -20055,10 +20255,14 @@
         <f>+'1_CC'!H21</f>
         <v>215340.02701247379</v>
       </c>
-    </row>
-    <row r="93" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M92" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="93" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B93">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>10</v>
       </c>
       <c r="C93" s="7" t="s">
@@ -20083,7 +20287,10 @@
         <f>+'1_CC'!I22</f>
         <v>20950080.661705784</v>
       </c>
-      <c r="I93" s="1"/>
+      <c r="I93" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J93" s="1">
         <f>+'1_CL'!AC18</f>
         <v>343341.33618595824</v>
@@ -20096,10 +20303,14 @@
         <f>+'1_CC'!H22</f>
         <v>261744.66170578444</v>
       </c>
-    </row>
-    <row r="94" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M93" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="94" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B94">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>9</v>
       </c>
       <c r="C94" s="7" t="s">
@@ -20124,7 +20335,10 @@
         <f>+'1_CC'!I23</f>
         <v>26735774.131052997</v>
       </c>
-      <c r="I94" s="1"/>
+      <c r="I94" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J94" s="1">
         <f>+'1_CL'!AC19</f>
         <v>832031.14012702927</v>
@@ -20137,10 +20351,14 @@
         <f>+'1_CC'!H23</f>
         <v>1088051.1310529986</v>
       </c>
-    </row>
-    <row r="95" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M94" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="95" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B95">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>8</v>
       </c>
       <c r="C95" s="7" t="s">
@@ -20165,7 +20383,10 @@
         <f>+'1_CC'!I24</f>
         <v>28112786.919644952</v>
       </c>
-      <c r="I95" s="1"/>
+      <c r="I95" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J95" s="1">
         <f>+'1_CL'!AC20</f>
         <v>1661641.4468988813</v>
@@ -20178,10 +20399,14 @@
         <f>+'1_CC'!H24</f>
         <v>1301322.9196449518</v>
       </c>
-    </row>
-    <row r="96" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M95" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="96" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B96">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>7</v>
       </c>
       <c r="C96" s="7" t="s">
@@ -20206,7 +20431,10 @@
         <f>+'1_CC'!I25</f>
         <v>24415375.979227304</v>
       </c>
-      <c r="I96" s="1"/>
+      <c r="I96" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J96" s="1">
         <f>+'1_CL'!AC21</f>
         <v>2608857.3940589502</v>
@@ -20219,10 +20447,14 @@
         <f>+'1_CC'!H25</f>
         <v>3016372.9792273026</v>
       </c>
+      <c r="M96" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
     </row>
     <row r="97" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B97">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>6</v>
       </c>
       <c r="C97" s="7" t="s">
@@ -20247,7 +20479,10 @@
         <f>+'1_CC'!I26</f>
         <v>41097760.732684806</v>
       </c>
-      <c r="I97" s="1"/>
+      <c r="I97" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J97" s="1">
         <f>+'1_CL'!AC22</f>
         <v>8321752.439681679</v>
@@ -20260,10 +20495,14 @@
         <f>+'1_CC'!H26</f>
         <v>7508497.7326848088</v>
       </c>
+      <c r="M97" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
     </row>
     <row r="98" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B98">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>5</v>
       </c>
       <c r="C98" s="7" t="s">
@@ -20288,7 +20527,10 @@
         <f>+'1_CC'!I27</f>
         <v>28807497.269866228</v>
       </c>
-      <c r="I98" s="1"/>
+      <c r="I98" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J98" s="1">
         <f>+'1_CL'!AC23</f>
         <v>8200379.2622825056</v>
@@ -20301,10 +20543,14 @@
         <f>+'1_CC'!H27</f>
         <v>7101712.269866229</v>
       </c>
+      <c r="M98" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
     </row>
     <row r="99" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B99">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>4</v>
       </c>
       <c r="C99" s="7" t="s">
@@ -20329,7 +20575,10 @@
         <f>+'1_CC'!I28</f>
         <v>30500846.83336778</v>
       </c>
-      <c r="I99" s="1"/>
+      <c r="I99" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J99" s="1">
         <f>+'1_CL'!AC24</f>
         <v>10399399.436663222</v>
@@ -20342,10 +20591,14 @@
         <f>+'1_CC'!H28</f>
         <v>13194752.83336778</v>
       </c>
+      <c r="M99" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
+      </c>
     </row>
     <row r="100" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B100">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>3</v>
       </c>
       <c r="C100" s="7" t="s">
@@ -20370,7 +20623,10 @@
         <f>+'1_CC'!I29</f>
         <v>27570818.173343755</v>
       </c>
-      <c r="I100" s="1"/>
+      <c r="I100" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J100" s="1">
         <f>+'1_CL'!AC25</f>
         <v>15289606.484099515</v>
@@ -20383,10 +20639,14 @@
         <f>+'1_CC'!H29</f>
         <v>12196356.173343755</v>
       </c>
+      <c r="M100" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
     </row>
     <row r="101" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B101">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>2</v>
       </c>
       <c r="C101" s="7" t="s">
@@ -20411,7 +20671,10 @@
         <f>+'1_CC'!I30</f>
         <v>21799017.90015018</v>
       </c>
-      <c r="I101" s="1"/>
+      <c r="I101" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J101" s="1">
         <f>+'1_CL'!AC26</f>
         <v>15731243.082726397</v>
@@ -20424,10 +20687,14 @@
         <f>+'1_CC'!H30</f>
         <v>12477183.90015018</v>
       </c>
+      <c r="M101" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>Chain Ladder</v>
+      </c>
     </row>
     <row r="102" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B102">
-        <f t="shared" si="30"/>
+        <f t="shared" si="32"/>
         <v>1</v>
       </c>
       <c r="C102" s="7" t="s">
@@ -20452,7 +20719,10 @@
         <f>+'1_CC'!I31</f>
         <v>30689191.735443387</v>
       </c>
-      <c r="I102" s="1"/>
+      <c r="I102" s="1" t="str">
+        <f t="shared" si="30"/>
+        <v>CC</v>
+      </c>
       <c r="J102" s="1">
         <f>+'1_CL'!AC27</f>
         <v>24566034.930802129</v>
@@ -20464,6 +20734,10 @@
       <c r="L102" s="79">
         <f>+'1_CC'!H31</f>
         <v>25539233.735443387</v>
+      </c>
+      <c r="M102" s="1" t="str">
+        <f t="shared" si="31"/>
+        <v>CC</v>
       </c>
     </row>
     <row r="108" spans="2:27" ht="26.25" x14ac:dyDescent="0.4">
@@ -20504,83 +20778,83 @@
         <v>2</v>
       </c>
       <c r="F110" s="10">
-        <f t="shared" ref="F110:AA110" si="31">+E110+1</f>
+        <f t="shared" ref="F110:AA110" si="33">+E110+1</f>
         <v>3</v>
       </c>
       <c r="G110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>4</v>
       </c>
       <c r="H110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>5</v>
       </c>
       <c r="I110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>6</v>
       </c>
       <c r="J110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>7</v>
       </c>
       <c r="K110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>8</v>
       </c>
       <c r="L110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>9</v>
       </c>
       <c r="M110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>10</v>
       </c>
       <c r="N110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>11</v>
       </c>
       <c r="O110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>12</v>
       </c>
       <c r="P110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>13</v>
       </c>
       <c r="Q110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>14</v>
       </c>
       <c r="R110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>15</v>
       </c>
       <c r="S110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>16</v>
       </c>
       <c r="T110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>17</v>
       </c>
       <c r="U110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>18</v>
       </c>
       <c r="V110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>19</v>
       </c>
       <c r="W110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>20</v>
       </c>
       <c r="X110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>21</v>
       </c>
       <c r="Y110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>22</v>
       </c>
       <c r="Z110" s="10">
@@ -20588,7 +20862,7 @@
         <v>23</v>
       </c>
       <c r="AA110" s="10">
-        <f t="shared" si="31"/>
+        <f t="shared" si="33"/>
         <v>24</v>
       </c>
     </row>
@@ -22765,70 +23039,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="155" t="s">
+      <c r="A1" s="147" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="155"/>
-      <c r="C1" s="155"/>
-      <c r="D1" s="155"/>
-      <c r="E1" s="155"/>
-      <c r="F1" s="155"/>
-      <c r="G1" s="155"/>
-      <c r="H1" s="155"/>
-      <c r="I1" s="155"/>
-      <c r="J1" s="155"/>
-      <c r="K1" s="155"/>
-      <c r="L1" s="155"/>
-      <c r="M1" s="155"/>
-      <c r="N1" s="155"/>
-      <c r="O1" s="155"/>
-      <c r="P1" s="155"/>
-      <c r="Q1" s="155"/>
-      <c r="R1" s="155"/>
-      <c r="S1" s="155"/>
-      <c r="T1" s="155"/>
-      <c r="U1" s="155"/>
-      <c r="V1" s="155"/>
-      <c r="W1" s="155"/>
-      <c r="X1" s="155"/>
-      <c r="Y1" s="155"/>
-      <c r="Z1" s="155"/>
-      <c r="AA1" s="155"/>
-      <c r="AB1" s="155"/>
-      <c r="AC1" s="155"/>
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+      <c r="D1" s="147"/>
+      <c r="E1" s="147"/>
+      <c r="F1" s="147"/>
+      <c r="G1" s="147"/>
+      <c r="H1" s="147"/>
+      <c r="I1" s="147"/>
+      <c r="J1" s="147"/>
+      <c r="K1" s="147"/>
+      <c r="L1" s="147"/>
+      <c r="M1" s="147"/>
+      <c r="N1" s="147"/>
+      <c r="O1" s="147"/>
+      <c r="P1" s="147"/>
+      <c r="Q1" s="147"/>
+      <c r="R1" s="147"/>
+      <c r="S1" s="147"/>
+      <c r="T1" s="147"/>
+      <c r="U1" s="147"/>
+      <c r="V1" s="147"/>
+      <c r="W1" s="147"/>
+      <c r="X1" s="147"/>
+      <c r="Y1" s="147"/>
+      <c r="Z1" s="147"/>
+      <c r="AA1" s="147"/>
+      <c r="AB1" s="147"/>
+      <c r="AC1" s="147"/>
     </row>
     <row r="2" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="156" t="s">
+      <c r="A2" s="148" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="156"/>
-      <c r="C2" s="156"/>
-      <c r="D2" s="156"/>
-      <c r="E2" s="156"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="156"/>
-      <c r="H2" s="156"/>
-      <c r="I2" s="156"/>
-      <c r="J2" s="156"/>
-      <c r="K2" s="156"/>
-      <c r="L2" s="156"/>
-      <c r="M2" s="156"/>
-      <c r="N2" s="156"/>
-      <c r="O2" s="156"/>
-      <c r="P2" s="156"/>
-      <c r="Q2" s="156"/>
-      <c r="R2" s="156"/>
-      <c r="S2" s="156"/>
-      <c r="T2" s="156"/>
-      <c r="U2" s="156"/>
-      <c r="V2" s="156"/>
-      <c r="W2" s="156"/>
-      <c r="X2" s="156"/>
-      <c r="Y2" s="156"/>
-      <c r="Z2" s="156"/>
-      <c r="AA2" s="156"/>
-      <c r="AB2" s="156"/>
-      <c r="AC2" s="156"/>
+      <c r="B2" s="148"/>
+      <c r="C2" s="148"/>
+      <c r="D2" s="148"/>
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="148"/>
+      <c r="H2" s="148"/>
+      <c r="I2" s="148"/>
+      <c r="J2" s="148"/>
+      <c r="K2" s="148"/>
+      <c r="L2" s="148"/>
+      <c r="M2" s="148"/>
+      <c r="N2" s="148"/>
+      <c r="O2" s="148"/>
+      <c r="P2" s="148"/>
+      <c r="Q2" s="148"/>
+      <c r="R2" s="148"/>
+      <c r="S2" s="148"/>
+      <c r="T2" s="148"/>
+      <c r="U2" s="148"/>
+      <c r="V2" s="148"/>
+      <c r="W2" s="148"/>
+      <c r="X2" s="148"/>
+      <c r="Y2" s="148"/>
+      <c r="Z2" s="148"/>
+      <c r="AA2" s="148"/>
+      <c r="AB2" s="148"/>
+      <c r="AC2" s="148"/>
     </row>
     <row r="3" spans="1:29" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
@@ -25652,10 +25926,10 @@
       <c r="AC30" s="38"/>
     </row>
     <row r="31" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="157" t="s">
+      <c r="A31" s="149" t="s">
         <v>151</v>
       </c>
-      <c r="B31" s="157"/>
+      <c r="B31" s="149"/>
       <c r="C31" s="81">
         <f>+C30*D31</f>
         <v>5.7701427721938954</v>
@@ -25756,10 +26030,10 @@
       <c r="AC31" s="38"/>
     </row>
     <row r="32" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="157" t="s">
+      <c r="A32" s="149" t="s">
         <v>152</v>
       </c>
-      <c r="B32" s="157"/>
+      <c r="B32" s="149"/>
       <c r="C32" s="64">
         <f>1/C31</f>
         <v>0.17330593704179437</v>
@@ -25860,34 +26134,34 @@
       <c r="AC32" s="38"/>
     </row>
     <row r="33" spans="1:29" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="158" t="s">
+      <c r="A33" s="150" t="s">
         <v>150</v>
       </c>
-      <c r="B33" s="159"/>
-      <c r="C33" s="159"/>
-      <c r="D33" s="159"/>
-      <c r="E33" s="159"/>
-      <c r="F33" s="159"/>
-      <c r="G33" s="159"/>
-      <c r="H33" s="159"/>
-      <c r="I33" s="159"/>
-      <c r="J33" s="159"/>
-      <c r="K33" s="159"/>
-      <c r="L33" s="159"/>
-      <c r="M33" s="159"/>
-      <c r="N33" s="159"/>
-      <c r="O33" s="159"/>
-      <c r="P33" s="159"/>
-      <c r="Q33" s="159"/>
-      <c r="R33" s="159"/>
-      <c r="S33" s="159"/>
-      <c r="T33" s="159"/>
-      <c r="U33" s="159"/>
-      <c r="V33" s="159"/>
-      <c r="W33" s="159"/>
-      <c r="X33" s="159"/>
-      <c r="Y33" s="159"/>
-      <c r="Z33" s="160"/>
+      <c r="B33" s="151"/>
+      <c r="C33" s="151"/>
+      <c r="D33" s="151"/>
+      <c r="E33" s="151"/>
+      <c r="F33" s="151"/>
+      <c r="G33" s="151"/>
+      <c r="H33" s="151"/>
+      <c r="I33" s="151"/>
+      <c r="J33" s="151"/>
+      <c r="K33" s="151"/>
+      <c r="L33" s="151"/>
+      <c r="M33" s="151"/>
+      <c r="N33" s="151"/>
+      <c r="O33" s="151"/>
+      <c r="P33" s="151"/>
+      <c r="Q33" s="151"/>
+      <c r="R33" s="151"/>
+      <c r="S33" s="151"/>
+      <c r="T33" s="151"/>
+      <c r="U33" s="151"/>
+      <c r="V33" s="151"/>
+      <c r="W33" s="151"/>
+      <c r="X33" s="151"/>
+      <c r="Y33" s="151"/>
+      <c r="Z33" s="152"/>
       <c r="AA33" s="45">
         <f>+SUM(AA4:AA27)</f>
         <v>502501456.85135591</v>
@@ -26836,15 +27110,15 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="161" t="s">
+      <c r="A32" s="153" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="161"/>
-      <c r="C32" s="161"/>
-      <c r="D32" s="161"/>
-      <c r="E32" s="161"/>
-      <c r="F32" s="161"/>
-      <c r="G32" s="161"/>
+      <c r="B32" s="153"/>
+      <c r="C32" s="153"/>
+      <c r="D32" s="153"/>
+      <c r="E32" s="153"/>
+      <c r="F32" s="153"/>
+      <c r="G32" s="153"/>
       <c r="H32" s="70">
         <f>SUM(H8:H31)</f>
         <v>83401231.980431959</v>
@@ -26872,30 +27146,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="162" t="s">
+      <c r="A1" s="154" t="s">
         <v>140</v>
       </c>
-      <c r="B1" s="162"/>
-      <c r="C1" s="162"/>
-      <c r="D1" s="162"/>
-      <c r="E1" s="162"/>
-      <c r="F1" s="162"/>
-      <c r="G1" s="162"/>
-      <c r="H1" s="162"/>
-      <c r="I1" s="162"/>
+      <c r="B1" s="154"/>
+      <c r="C1" s="154"/>
+      <c r="D1" s="154"/>
+      <c r="E1" s="154"/>
+      <c r="F1" s="154"/>
+      <c r="G1" s="154"/>
+      <c r="H1" s="154"/>
+      <c r="I1" s="154"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="163" t="s">
+      <c r="A2" s="155" t="s">
         <v>141</v>
       </c>
-      <c r="B2" s="163"/>
-      <c r="C2" s="163"/>
-      <c r="D2" s="163"/>
-      <c r="E2" s="163"/>
-      <c r="F2" s="163"/>
-      <c r="G2" s="163"/>
-      <c r="H2" s="163"/>
-      <c r="I2" s="163"/>
+      <c r="B2" s="155"/>
+      <c r="C2" s="155"/>
+      <c r="D2" s="155"/>
+      <c r="E2" s="155"/>
+      <c r="F2" s="155"/>
+      <c r="G2" s="155"/>
+      <c r="H2" s="155"/>
+      <c r="I2" s="155"/>
     </row>
     <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -27852,14 +28126,14 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="164" t="s">
+      <c r="A32" s="156" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="165"/>
-      <c r="C32" s="165"/>
-      <c r="D32" s="165"/>
-      <c r="E32" s="165"/>
-      <c r="F32" s="166"/>
+      <c r="B32" s="157"/>
+      <c r="C32" s="157"/>
+      <c r="D32" s="157"/>
+      <c r="E32" s="157"/>
+      <c r="F32" s="158"/>
       <c r="G32" s="80">
         <f>SUM(G8:G31)</f>
         <v>747315102.91086709</v>
@@ -27899,28 +28173,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="146" t="s">
+      <c r="B1" s="163" t="s">
         <v>153</v>
       </c>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
+      <c r="C1" s="163"/>
+      <c r="D1" s="163"/>
+      <c r="E1" s="163"/>
+      <c r="F1" s="163"/>
+      <c r="G1" s="163"/>
+      <c r="H1" s="163"/>
+      <c r="I1" s="163"/>
     </row>
     <row r="2" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="147" t="s">
+      <c r="B2" s="164" t="s">
         <v>154</v>
       </c>
-      <c r="C2" s="147"/>
-      <c r="D2" s="147"/>
-      <c r="E2" s="147"/>
-      <c r="F2" s="147"/>
-      <c r="G2" s="147"/>
-      <c r="H2" s="147"/>
-      <c r="I2" s="147"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="164"/>
+      <c r="G2" s="164"/>
+      <c r="H2" s="164"/>
+      <c r="I2" s="164"/>
       <c r="N2" s="28" t="s">
         <v>245</v>
       </c>
@@ -27931,12 +28205,12 @@
       </c>
     </row>
     <row r="4" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="148" t="s">
+      <c r="B4" s="161" t="s">
         <v>155</v>
       </c>
-      <c r="C4" s="148"/>
-      <c r="D4" s="148"/>
-      <c r="E4" s="148"/>
+      <c r="C4" s="161"/>
+      <c r="D4" s="161"/>
+      <c r="E4" s="161"/>
       <c r="I4" s="28" t="s">
         <v>245</v>
       </c>
@@ -27949,14 +28223,14 @@
         <f>'1_CL'!AC33</f>
         <v>88287625.851355985</v>
       </c>
-      <c r="D5" s="149" t="s">
+      <c r="D5" s="165" t="s">
         <v>157</v>
       </c>
-      <c r="E5" s="149"/>
-      <c r="F5" s="149"/>
-      <c r="G5" s="149"/>
-      <c r="H5" s="149"/>
-      <c r="I5" s="149"/>
+      <c r="E5" s="165"/>
+      <c r="F5" s="165"/>
+      <c r="G5" s="165"/>
+      <c r="H5" s="165"/>
+      <c r="I5" s="165"/>
     </row>
     <row r="6" spans="2:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="83" t="s">
@@ -27966,14 +28240,14 @@
         <f>IF(I4="Anual",Triangulo1!E4, POWER(1+Triangulo1!E4,0.25)-1)</f>
         <v>1.4673846168659299E-2</v>
       </c>
-      <c r="D6" s="149" t="s">
+      <c r="D6" s="165" t="s">
         <v>159</v>
       </c>
-      <c r="E6" s="149"/>
-      <c r="F6" s="149"/>
-      <c r="G6" s="149"/>
-      <c r="H6" s="149"/>
-      <c r="I6" s="149"/>
+      <c r="E6" s="165"/>
+      <c r="F6" s="165"/>
+      <c r="G6" s="165"/>
+      <c r="H6" s="165"/>
+      <c r="I6" s="165"/>
       <c r="J6" s="86">
         <v>0.04</v>
       </c>
@@ -27985,14 +28259,14 @@
       <c r="C7" s="85">
         <v>0.01</v>
       </c>
-      <c r="D7" s="149" t="s">
+      <c r="D7" s="165" t="s">
         <v>161</v>
       </c>
-      <c r="E7" s="149"/>
-      <c r="F7" s="149"/>
-      <c r="G7" s="149"/>
-      <c r="H7" s="149"/>
-      <c r="I7" s="149"/>
+      <c r="E7" s="165"/>
+      <c r="F7" s="165"/>
+      <c r="G7" s="165"/>
+      <c r="H7" s="165"/>
+      <c r="I7" s="165"/>
     </row>
     <row r="8" spans="2:14" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="83" t="s">
@@ -28001,26 +28275,26 @@
       <c r="C8" s="85">
         <v>0.4</v>
       </c>
-      <c r="D8" s="149" t="s">
+      <c r="D8" s="165" t="s">
         <v>163</v>
       </c>
-      <c r="E8" s="149"/>
-      <c r="F8" s="149"/>
-      <c r="G8" s="149"/>
-      <c r="H8" s="149"/>
-      <c r="I8" s="149"/>
+      <c r="E8" s="165"/>
+      <c r="F8" s="165"/>
+      <c r="G8" s="165"/>
+      <c r="H8" s="165"/>
+      <c r="I8" s="165"/>
     </row>
     <row r="10" spans="2:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="148" t="s">
+      <c r="B10" s="161" t="s">
         <v>164</v>
       </c>
-      <c r="C10" s="148"/>
-      <c r="D10" s="148"/>
-      <c r="E10" s="148"/>
-      <c r="F10" s="148"/>
-      <c r="G10" s="148"/>
-      <c r="H10" s="148"/>
-      <c r="I10" s="148"/>
+      <c r="C10" s="161"/>
+      <c r="D10" s="161"/>
+      <c r="E10" s="161"/>
+      <c r="F10" s="161"/>
+      <c r="G10" s="161"/>
+      <c r="H10" s="161"/>
+      <c r="I10" s="161"/>
     </row>
     <row r="11" spans="2:14" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="87" t="s">
@@ -29006,16 +29280,16 @@
       </c>
     </row>
     <row r="38" spans="2:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="150" t="s">
+      <c r="B38" s="166" t="s">
         <v>173</v>
       </c>
-      <c r="C38" s="150"/>
-      <c r="D38" s="150"/>
-      <c r="E38" s="150"/>
-      <c r="F38" s="150"/>
-      <c r="G38" s="150"/>
-      <c r="H38" s="150"/>
-      <c r="I38" s="150"/>
+      <c r="C38" s="166"/>
+      <c r="D38" s="166"/>
+      <c r="E38" s="166"/>
+      <c r="F38" s="166"/>
+      <c r="G38" s="166"/>
+      <c r="H38" s="166"/>
+      <c r="I38" s="166"/>
     </row>
     <row r="39" spans="2:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="101" t="s">
@@ -29028,15 +29302,15 @@
       <c r="D39" s="103" t="s">
         <v>175</v>
       </c>
-      <c r="E39" s="144" t="s">
+      <c r="E39" s="162" t="s">
         <v>176</v>
       </c>
-      <c r="F39" s="144"/>
-      <c r="G39" s="144"/>
-      <c r="H39" s="145" t="s">
+      <c r="F39" s="162"/>
+      <c r="G39" s="162"/>
+      <c r="H39" s="160" t="s">
         <v>247</v>
       </c>
-      <c r="I39" s="145"/>
+      <c r="I39" s="160"/>
     </row>
     <row r="40" spans="2:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="2:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -29050,15 +29324,15 @@
       <c r="D41" s="103" t="s">
         <v>175</v>
       </c>
-      <c r="E41" s="144" t="s">
+      <c r="E41" s="162" t="s">
         <v>178</v>
       </c>
-      <c r="F41" s="144"/>
-      <c r="G41" s="144"/>
-      <c r="H41" s="145" t="s">
+      <c r="F41" s="162"/>
+      <c r="G41" s="162"/>
+      <c r="H41" s="160" t="s">
         <v>248</v>
       </c>
-      <c r="I41" s="145"/>
+      <c r="I41" s="160"/>
       <c r="J41" s="100"/>
     </row>
     <row r="42" spans="2:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -29071,28 +29345,28 @@
         <v>2.1040038751255778</v>
       </c>
       <c r="D43" s="106"/>
-      <c r="E43" s="151" t="s">
+      <c r="E43" s="159" t="s">
         <v>180</v>
       </c>
-      <c r="F43" s="151"/>
-      <c r="G43" s="151"/>
-      <c r="H43" s="145" t="s">
+      <c r="F43" s="159"/>
+      <c r="G43" s="159"/>
+      <c r="H43" s="160" t="s">
         <v>181</v>
       </c>
-      <c r="I43" s="145"/>
+      <c r="I43" s="160"/>
     </row>
     <row r="44" spans="2:11" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="148" t="s">
+      <c r="B46" s="161" t="s">
         <v>182</v>
       </c>
-      <c r="C46" s="148"/>
-      <c r="D46" s="148"/>
-      <c r="E46" s="148"/>
-      <c r="F46" s="148"/>
-      <c r="G46" s="148"/>
-      <c r="H46" s="148"/>
-      <c r="I46" s="148"/>
+      <c r="C46" s="161"/>
+      <c r="D46" s="161"/>
+      <c r="E46" s="161"/>
+      <c r="F46" s="161"/>
+      <c r="G46" s="161"/>
+      <c r="H46" s="161"/>
+      <c r="I46" s="161"/>
     </row>
     <row r="47" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="107" t="s">
@@ -29239,22 +29513,22 @@
   </sheetData>
   <dataConsolidate/>
   <mergeCells count="16">
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="B46:I46"/>
-    <mergeCell ref="E41:G41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="D6:I6"/>
     <mergeCell ref="D7:I7"/>
     <mergeCell ref="D8:I8"/>
     <mergeCell ref="B10:I10"/>
     <mergeCell ref="B38:I38"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="H39:I39"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="D6:I6"/>
+    <mergeCell ref="E43:G43"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="E41:G41"/>
+    <mergeCell ref="H41:I41"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I4" xr:uid="{BD7165A2-6146-4907-BCCF-5174555EA24E}">
@@ -29325,34 +29599,34 @@
       <c r="AA1" s="169"/>
     </row>
     <row r="3" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A3" s="148" t="s">
+      <c r="A3" s="161" t="s">
         <v>198</v>
       </c>
-      <c r="B3" s="148"/>
-      <c r="C3" s="148"/>
-      <c r="D3" s="148"/>
-      <c r="E3" s="148"/>
-      <c r="F3" s="148"/>
-      <c r="G3" s="148"/>
-      <c r="H3" s="148"/>
-      <c r="I3" s="148"/>
-      <c r="J3" s="148"/>
-      <c r="K3" s="148"/>
-      <c r="L3" s="148"/>
-      <c r="M3" s="148"/>
-      <c r="N3" s="148"/>
-      <c r="O3" s="148"/>
-      <c r="P3" s="148"/>
-      <c r="Q3" s="148"/>
-      <c r="R3" s="148"/>
-      <c r="S3" s="148"/>
-      <c r="T3" s="148"/>
-      <c r="U3" s="148"/>
-      <c r="V3" s="148"/>
-      <c r="W3" s="148"/>
-      <c r="X3" s="148"/>
-      <c r="Y3" s="148"/>
-      <c r="Z3" s="148"/>
+      <c r="B3" s="161"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
+      <c r="E3" s="161"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
+      <c r="J3" s="161"/>
+      <c r="K3" s="161"/>
+      <c r="L3" s="161"/>
+      <c r="M3" s="161"/>
+      <c r="N3" s="161"/>
+      <c r="O3" s="161"/>
+      <c r="P3" s="161"/>
+      <c r="Q3" s="161"/>
+      <c r="R3" s="161"/>
+      <c r="S3" s="161"/>
+      <c r="T3" s="161"/>
+      <c r="U3" s="161"/>
+      <c r="V3" s="161"/>
+      <c r="W3" s="161"/>
+      <c r="X3" s="161"/>
+      <c r="Y3" s="161"/>
+      <c r="Z3" s="161"/>
     </row>
     <row r="4" spans="1:51" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="107" t="s">
@@ -33417,33 +33691,33 @@
       </c>
     </row>
     <row r="31" spans="1:51" x14ac:dyDescent="0.25">
-      <c r="A31" s="148" t="s">
+      <c r="A31" s="161" t="s">
         <v>207</v>
       </c>
-      <c r="B31" s="148"/>
-      <c r="C31" s="148"/>
-      <c r="D31" s="148"/>
-      <c r="E31" s="148"/>
-      <c r="F31" s="148"/>
-      <c r="G31" s="148"/>
-      <c r="H31" s="148"/>
-      <c r="I31" s="148"/>
-      <c r="J31" s="148"/>
-      <c r="K31" s="148"/>
-      <c r="L31" s="148"/>
-      <c r="M31" s="148"/>
-      <c r="N31" s="148"/>
-      <c r="O31" s="148"/>
-      <c r="P31" s="148"/>
-      <c r="Q31" s="148"/>
-      <c r="R31" s="148"/>
-      <c r="S31" s="148"/>
-      <c r="T31" s="148"/>
-      <c r="U31" s="148"/>
-      <c r="V31" s="148"/>
-      <c r="W31" s="148"/>
-      <c r="X31" s="148"/>
-      <c r="Y31" s="148"/>
+      <c r="B31" s="161"/>
+      <c r="C31" s="161"/>
+      <c r="D31" s="161"/>
+      <c r="E31" s="161"/>
+      <c r="F31" s="161"/>
+      <c r="G31" s="161"/>
+      <c r="H31" s="161"/>
+      <c r="I31" s="161"/>
+      <c r="J31" s="161"/>
+      <c r="K31" s="161"/>
+      <c r="L31" s="161"/>
+      <c r="M31" s="161"/>
+      <c r="N31" s="161"/>
+      <c r="O31" s="161"/>
+      <c r="P31" s="161"/>
+      <c r="Q31" s="161"/>
+      <c r="R31" s="161"/>
+      <c r="S31" s="161"/>
+      <c r="T31" s="161"/>
+      <c r="U31" s="161"/>
+      <c r="V31" s="161"/>
+      <c r="W31" s="161"/>
+      <c r="X31" s="161"/>
+      <c r="Y31" s="161"/>
     </row>
     <row r="32" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A32" s="107" t="s">
@@ -38556,50 +38830,62 @@
       <c r="D8" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="H8" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="9" spans="3:27" x14ac:dyDescent="0.25">
       <c r="D9" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="H9" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="10" spans="3:27" x14ac:dyDescent="0.25">
       <c r="D10" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H10" t="s">
+        <v>258</v>
+      </c>
     </row>
     <row r="11" spans="3:27" x14ac:dyDescent="0.25">
       <c r="D11" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="H11" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="13" spans="3:27" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="C13" s="152" t="s">
+      <c r="C13" s="144" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="152"/>
-      <c r="E13" s="152"/>
-      <c r="F13" s="152"/>
-      <c r="G13" s="152"/>
-      <c r="H13" s="152"/>
-      <c r="I13" s="152"/>
-      <c r="J13" s="152"/>
-      <c r="K13" s="152"/>
-      <c r="L13" s="152"/>
-      <c r="M13" s="152"/>
-      <c r="N13" s="152"/>
-      <c r="O13" s="152"/>
-      <c r="P13" s="152"/>
-      <c r="Q13" s="152"/>
-      <c r="R13" s="152"/>
-      <c r="S13" s="152"/>
-      <c r="T13" s="152"/>
-      <c r="U13" s="152"/>
-      <c r="V13" s="152"/>
-      <c r="W13" s="152"/>
-      <c r="X13" s="152"/>
-      <c r="Y13" s="152"/>
-      <c r="Z13" s="152"/>
-      <c r="AA13" s="152"/>
+      <c r="D13" s="144"/>
+      <c r="E13" s="144"/>
+      <c r="F13" s="144"/>
+      <c r="G13" s="144"/>
+      <c r="H13" s="144"/>
+      <c r="I13" s="144"/>
+      <c r="J13" s="144"/>
+      <c r="K13" s="144"/>
+      <c r="L13" s="144"/>
+      <c r="M13" s="144"/>
+      <c r="N13" s="144"/>
+      <c r="O13" s="144"/>
+      <c r="P13" s="144"/>
+      <c r="Q13" s="144"/>
+      <c r="R13" s="144"/>
+      <c r="S13" s="144"/>
+      <c r="T13" s="144"/>
+      <c r="U13" s="144"/>
+      <c r="V13" s="144"/>
+      <c r="W13" s="144"/>
+      <c r="X13" s="144"/>
+      <c r="Y13" s="144"/>
+      <c r="Z13" s="144"/>
+      <c r="AA13" s="144"/>
     </row>
     <row r="15" spans="3:27" x14ac:dyDescent="0.25">
       <c r="D15" s="11">
@@ -40597,33 +40883,33 @@
       <c r="AA41" s="3"/>
     </row>
     <row r="42" spans="3:27" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="C42" s="152" t="s">
+      <c r="C42" s="144" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="152"/>
-      <c r="E42" s="152"/>
-      <c r="F42" s="152"/>
-      <c r="G42" s="152"/>
-      <c r="H42" s="152"/>
-      <c r="I42" s="152"/>
-      <c r="J42" s="152"/>
-      <c r="K42" s="152"/>
-      <c r="L42" s="152"/>
-      <c r="M42" s="152"/>
-      <c r="N42" s="152"/>
-      <c r="O42" s="152"/>
-      <c r="P42" s="152"/>
-      <c r="Q42" s="152"/>
-      <c r="R42" s="152"/>
-      <c r="S42" s="152"/>
-      <c r="T42" s="152"/>
-      <c r="U42" s="152"/>
-      <c r="V42" s="152"/>
-      <c r="W42" s="152"/>
-      <c r="X42" s="152"/>
-      <c r="Y42" s="152"/>
-      <c r="Z42" s="152"/>
-      <c r="AA42" s="152"/>
+      <c r="D42" s="144"/>
+      <c r="E42" s="144"/>
+      <c r="F42" s="144"/>
+      <c r="G42" s="144"/>
+      <c r="H42" s="144"/>
+      <c r="I42" s="144"/>
+      <c r="J42" s="144"/>
+      <c r="K42" s="144"/>
+      <c r="L42" s="144"/>
+      <c r="M42" s="144"/>
+      <c r="N42" s="144"/>
+      <c r="O42" s="144"/>
+      <c r="P42" s="144"/>
+      <c r="Q42" s="144"/>
+      <c r="R42" s="144"/>
+      <c r="S42" s="144"/>
+      <c r="T42" s="144"/>
+      <c r="U42" s="144"/>
+      <c r="V42" s="144"/>
+      <c r="W42" s="144"/>
+      <c r="X42" s="144"/>
+      <c r="Y42" s="144"/>
+      <c r="Z42" s="144"/>
+      <c r="AA42" s="144"/>
     </row>
     <row r="43" spans="3:27" x14ac:dyDescent="0.25">
       <c r="C43" s="11">
@@ -42640,18 +42926,18 @@
       <c r="J75" s="1"/>
     </row>
     <row r="76" spans="2:27" x14ac:dyDescent="0.25">
-      <c r="F76" s="153" t="s">
+      <c r="F76" s="145" t="s">
         <v>36</v>
       </c>
-      <c r="G76" s="153"/>
-      <c r="H76" s="153"/>
-      <c r="I76" s="153"/>
-      <c r="J76" s="154" t="s">
+      <c r="G76" s="145"/>
+      <c r="H76" s="145"/>
+      <c r="I76" s="145"/>
+      <c r="J76" s="146" t="s">
         <v>37</v>
       </c>
-      <c r="K76" s="154"/>
-      <c r="L76" s="154"/>
-      <c r="M76" s="154"/>
+      <c r="K76" s="146"/>
+      <c r="L76" s="146"/>
+      <c r="M76" s="146"/>
     </row>
     <row r="77" spans="2:27" x14ac:dyDescent="0.25">
       <c r="D77" s="4" t="s">
@@ -42711,7 +42997,10 @@
         <f>'2_CC'!I8</f>
         <v>5814528</v>
       </c>
-      <c r="I78" s="1"/>
+      <c r="I78" s="1" t="str">
+        <f>IF(MAX(F78:H78)=F78,"Chain Ladder",IF(MAX(F78:H78)=G78,"BF","CC"))</f>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J78" s="1">
         <f>'2_CL'!AC4</f>
         <v>0</v>
@@ -42723,6 +43012,10 @@
       <c r="L78" s="5">
         <f>'2_CC'!H8</f>
         <v>0</v>
+      </c>
+      <c r="M78" s="1" t="str">
+        <f>IF(MAX(J78:L78)=J78,"Chain Ladder",IF(MAX(J78:L78)=K78,"BF","CC"))</f>
+        <v>Chain Ladder</v>
       </c>
     </row>
     <row r="79" spans="2:27" x14ac:dyDescent="0.25">
@@ -42752,7 +43045,10 @@
         <f>'2_CC'!I9</f>
         <v>7995875.6912902556</v>
       </c>
-      <c r="I79" s="1"/>
+      <c r="I79" s="1" t="str">
+        <f t="shared" ref="I79:I101" si="45">IF(MAX(F79:H79)=F79,"Chain Ladder",IF(MAX(F79:H79)=G79,"BF","CC"))</f>
+        <v>BF</v>
+      </c>
       <c r="J79" s="1">
         <f>'2_CL'!AC5</f>
         <v>1.3751546777784824</v>
@@ -42765,10 +43061,14 @@
         <f>'2_CC'!H9</f>
         <v>1.6912902551866109</v>
       </c>
+      <c r="M79" s="1" t="str">
+        <f t="shared" ref="M79:M101" si="46">IF(MAX(J79:L79)=J79,"Chain Ladder",IF(MAX(J79:L79)=K79,"BF","CC"))</f>
+        <v>BF</v>
+      </c>
     </row>
     <row r="80" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B80">
-        <f t="shared" ref="B80:B101" si="45">+B79-1</f>
+        <f t="shared" ref="B80:B101" si="47">+B79-1</f>
         <v>22</v>
       </c>
       <c r="C80" s="9" t="s">
@@ -42793,7 +43093,10 @@
         <f>'2_CC'!I10</f>
         <v>4710880.6892100703</v>
       </c>
-      <c r="I80" s="1"/>
+      <c r="I80" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>BF</v>
+      </c>
       <c r="J80" s="1">
         <f>'2_CL'!AC6</f>
         <v>5.926850626245141</v>
@@ -42806,10 +43109,14 @@
         <f>'2_CC'!H10</f>
         <v>10.689210070358609</v>
       </c>
-    </row>
-    <row r="81" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M80" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>BF</v>
+      </c>
+    </row>
+    <row r="81" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B81">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>21</v>
       </c>
       <c r="C81" s="9" t="s">
@@ -42834,7 +43141,10 @@
         <f>'2_CC'!I11</f>
         <v>5046132.8632867727</v>
       </c>
-      <c r="I81" s="1"/>
+      <c r="I81" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J81" s="1">
         <f>'2_CL'!AC7</f>
         <v>12.615014017559588</v>
@@ -42847,10 +43157,14 @@
         <f>'2_CC'!H11</f>
         <v>9.8632867732058713</v>
       </c>
-    </row>
-    <row r="82" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M81" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="82" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B82">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>20</v>
       </c>
       <c r="C82" s="9" t="s">
@@ -42875,7 +43189,10 @@
         <f>'2_CC'!I12</f>
         <v>4612006.9662562022</v>
       </c>
-      <c r="I82" s="1"/>
+      <c r="I82" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J82" s="1">
         <f>'2_CL'!AC8</f>
         <v>-15.671818740665913</v>
@@ -42888,10 +43205,14 @@
         <f>'2_CC'!H12</f>
         <v>-28.033743797346361</v>
       </c>
-    </row>
-    <row r="83" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M82" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="83" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B83">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>19</v>
       </c>
       <c r="C83" s="9" t="s">
@@ -42916,7 +43237,10 @@
         <f>'2_CC'!I13</f>
         <v>2490242.3188707144</v>
       </c>
-      <c r="I83" s="1"/>
+      <c r="I83" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>BF</v>
+      </c>
       <c r="J83" s="1">
         <f>'2_CL'!AC9</f>
         <v>-81.718273874372244</v>
@@ -42929,10 +43253,14 @@
         <f>'2_CC'!H13</f>
         <v>14.318870714205902</v>
       </c>
-    </row>
-    <row r="84" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M83" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>BF</v>
+      </c>
+    </row>
+    <row r="84" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B84">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>18</v>
       </c>
       <c r="C84" s="9" t="s">
@@ -42957,7 +43285,10 @@
         <f>'2_CC'!I14</f>
         <v>2642618.2606514543</v>
       </c>
-      <c r="I84" s="1"/>
+      <c r="I84" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>BF</v>
+      </c>
       <c r="J84" s="1">
         <f>'2_CL'!AC10</f>
         <v>-345.55584763502702</v>
@@ -42970,10 +43301,14 @@
         <f>'2_CC'!H14</f>
         <v>337.26065145448621</v>
       </c>
-    </row>
-    <row r="85" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M84" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>BF</v>
+      </c>
+    </row>
+    <row r="85" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B85">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>17</v>
       </c>
       <c r="C85" s="9" t="s">
@@ -42998,7 +43333,10 @@
         <f>'2_CC'!I15</f>
         <v>6538427.3159776395</v>
       </c>
-      <c r="I85" s="1"/>
+      <c r="I85" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>CC</v>
+      </c>
       <c r="J85" s="1">
         <f>'2_CL'!AC11</f>
         <v>-1613.9375442489982</v>
@@ -43011,10 +43349,14 @@
         <f>'2_CC'!H15</f>
         <v>-457.68402236072637</v>
       </c>
-    </row>
-    <row r="86" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M85" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="86" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B86">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>16</v>
       </c>
       <c r="C86" s="9" t="s">
@@ -43039,7 +43381,10 @@
         <f>'2_CC'!I16</f>
         <v>6034807.1530441185</v>
       </c>
-      <c r="I86" s="1"/>
+      <c r="I86" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J86" s="1">
         <f>'2_CL'!AC12</f>
         <v>-2143.6379576781765</v>
@@ -43052,10 +43397,14 @@
         <f>'2_CC'!H16</f>
         <v>-2490.8469558811776</v>
       </c>
-    </row>
-    <row r="87" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M86" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="87" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B87">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>15</v>
       </c>
       <c r="C87" s="9" t="s">
@@ -43080,7 +43429,10 @@
         <f>'2_CC'!I17</f>
         <v>4348809.2535007121</v>
       </c>
-      <c r="I87" s="1"/>
+      <c r="I87" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J87" s="1">
         <f>'2_CL'!AC13</f>
         <v>-3331.3643750632182</v>
@@ -43093,10 +43445,14 @@
         <f>'2_CC'!H17</f>
         <v>-5603.7464992876166</v>
       </c>
-    </row>
-    <row r="88" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M87" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="88" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B88">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>14</v>
       </c>
       <c r="C88" s="9" t="s">
@@ -43121,7 +43477,10 @@
         <f>'2_CC'!I18</f>
         <v>4287581.1438070331</v>
       </c>
-      <c r="I88" s="1"/>
+      <c r="I88" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>BF</v>
+      </c>
       <c r="J88" s="1">
         <f>'2_CL'!AC14</f>
         <v>-6899.9200591864064</v>
@@ -43134,10 +43493,14 @@
         <f>'2_CC'!H18</f>
         <v>2928.1438070333552</v>
       </c>
-    </row>
-    <row r="89" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M88" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>BF</v>
+      </c>
+    </row>
+    <row r="89" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B89">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>13</v>
       </c>
       <c r="C89" s="9" t="s">
@@ -43162,7 +43525,10 @@
         <f>'2_CC'!I19</f>
         <v>7261250.4508135021</v>
       </c>
-      <c r="I89" s="1"/>
+      <c r="I89" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>CC</v>
+      </c>
       <c r="J89" s="1">
         <f>'2_CL'!AC15</f>
         <v>-26598.651411228813</v>
@@ -43175,10 +43541,14 @@
         <f>'2_CC'!H19</f>
         <v>-5590.5491864979049</v>
       </c>
-    </row>
-    <row r="90" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M89" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="90" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B90">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>12</v>
       </c>
       <c r="C90" s="9" t="s">
@@ -43203,7 +43573,10 @@
         <f>'2_CC'!I20</f>
         <v>5787262.3223339217</v>
       </c>
-      <c r="I90" s="1"/>
+      <c r="I90" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J90" s="1">
         <f>'2_CL'!AC16</f>
         <v>-43970.389721929096</v>
@@ -43216,10 +43589,14 @@
         <f>'2_CC'!H20</f>
         <v>-57505.677666078154</v>
       </c>
-    </row>
-    <row r="91" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M90" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="91" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B91">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>11</v>
       </c>
       <c r="C91" s="9" t="s">
@@ -43244,7 +43621,10 @@
         <f>'2_CC'!I21</f>
         <v>5067372.2213276364</v>
       </c>
-      <c r="I91" s="1"/>
+      <c r="I91" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J91" s="1">
         <f>'2_CL'!AC17</f>
         <v>-79335.360579818487</v>
@@ -43257,10 +43637,14 @@
         <f>'2_CC'!H21</f>
         <v>-104432.77867236319</v>
       </c>
-    </row>
-    <row r="92" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M91" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="92" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B92">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>10</v>
       </c>
       <c r="C92" s="9" t="s">
@@ -43285,7 +43669,10 @@
         <f>'2_CC'!I22</f>
         <v>2247700.0177094759</v>
       </c>
-      <c r="I92" s="1"/>
+      <c r="I92" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J92" s="1">
         <f>'2_CL'!AC18</f>
         <v>-80563.884190600831</v>
@@ -43298,10 +43685,14 @@
         <f>'2_CC'!H22</f>
         <v>-225424.98229052406</v>
       </c>
-    </row>
-    <row r="93" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M92" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="93" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B93">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>9</v>
       </c>
       <c r="C93" s="9" t="s">
@@ -43326,7 +43717,10 @@
         <f>'2_CC'!I23</f>
         <v>12892536.045075754</v>
       </c>
-      <c r="I93" s="1"/>
+      <c r="I93" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>CC</v>
+      </c>
       <c r="J93" s="1">
         <f>'2_CL'!AC19</f>
         <v>-724781.94354595616</v>
@@ -43339,10 +43733,14 @@
         <f>'2_CC'!H23</f>
         <v>-479076.95492424554</v>
       </c>
-    </row>
-    <row r="94" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M93" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>CC</v>
+      </c>
+    </row>
+    <row r="94" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B94">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>8</v>
       </c>
       <c r="C94" s="9" t="s">
@@ -43367,7 +43765,10 @@
         <f>'2_CC'!I24</f>
         <v>11253824.557890851</v>
       </c>
-      <c r="I94" s="1"/>
+      <c r="I94" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J94" s="1">
         <f>'2_CL'!AC20</f>
         <v>-949684.63453150913</v>
@@ -43380,10 +43781,14 @@
         <f>'2_CC'!H24</f>
         <v>-1168872.4421091494</v>
       </c>
-    </row>
-    <row r="95" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M94" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="95" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B95">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>7</v>
       </c>
       <c r="C95" s="9" t="s">
@@ -43408,7 +43813,10 @@
         <f>'2_CC'!I25</f>
         <v>9364066.5690304488</v>
       </c>
-      <c r="I95" s="1"/>
+      <c r="I95" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J95" s="1">
         <f>'2_CL'!AC21</f>
         <v>-1069760.5577581134</v>
@@ -43421,10 +43829,14 @@
         <f>'2_CC'!H25</f>
         <v>-1204562.4309695503</v>
       </c>
-    </row>
-    <row r="96" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="M95" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
+    </row>
+    <row r="96" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B96">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>6</v>
       </c>
       <c r="C96" s="9" t="s">
@@ -43449,7 +43861,10 @@
         <f>'2_CC'!I26</f>
         <v>22015501.506653816</v>
       </c>
-      <c r="I96" s="1"/>
+      <c r="I96" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J96" s="1">
         <f>'2_CL'!AC22</f>
         <v>-3456342.6733150929</v>
@@ -43462,10 +43877,14 @@
         <f>'2_CC'!H26</f>
         <v>-3577529.4933461864</v>
       </c>
+      <c r="M96" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
     </row>
     <row r="97" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B97">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>5</v>
       </c>
       <c r="C97" s="9" t="s">
@@ -43490,7 +43909,10 @@
         <f>'2_CC'!I27</f>
         <v>11680729.405287839</v>
       </c>
-      <c r="I97" s="1"/>
+      <c r="I97" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J97" s="1">
         <f>'2_CL'!AC23</f>
         <v>-2281110.0632403623</v>
@@ -43503,10 +43925,14 @@
         <f>'2_CC'!H27</f>
         <v>-2594420.5947121605</v>
       </c>
+      <c r="M97" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
     </row>
     <row r="98" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B98">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>4</v>
       </c>
       <c r="C98" s="9" t="s">
@@ -43531,7 +43957,10 @@
         <f>'2_CC'!I28</f>
         <v>9549194.5684155077</v>
       </c>
-      <c r="I98" s="1"/>
+      <c r="I98" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>Chain Ladder</v>
+      </c>
       <c r="J98" s="1">
         <f>'2_CL'!AC24</f>
         <v>-2481881.0143102854</v>
@@ -43544,10 +43973,14 @@
         <f>'2_CC'!H28</f>
         <v>-3186000.4315844928</v>
       </c>
+      <c r="M98" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>Chain Ladder</v>
+      </c>
     </row>
     <row r="99" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B99">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>3</v>
       </c>
       <c r="C99" s="9" t="s">
@@ -43572,7 +44005,10 @@
         <f>'2_CC'!I29</f>
         <v>10581008.854659371</v>
       </c>
-      <c r="I99" s="1"/>
+      <c r="I99" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>CC</v>
+      </c>
       <c r="J99" s="1">
         <f>'2_CL'!AC25</f>
         <v>-1394804.8884851448</v>
@@ -43585,10 +44021,14 @@
         <f>'2_CC'!H29</f>
         <v>-696864.14534062811</v>
       </c>
+      <c r="M99" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>CC</v>
+      </c>
     </row>
     <row r="100" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B100">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>2</v>
       </c>
       <c r="C100" s="9" t="s">
@@ -43613,7 +44053,10 @@
         <f>'2_CC'!I30</f>
         <v>8433522.989737682</v>
       </c>
-      <c r="I100" s="1"/>
+      <c r="I100" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>CC</v>
+      </c>
       <c r="J100" s="1">
         <f>'2_CL'!AC26</f>
         <v>-1632729.8086488377</v>
@@ -43626,10 +44069,14 @@
         <f>'2_CC'!H30</f>
         <v>-888311.01026231807</v>
       </c>
+      <c r="M100" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>CC</v>
+      </c>
     </row>
     <row r="101" spans="2:27" x14ac:dyDescent="0.25">
       <c r="B101">
-        <f t="shared" si="45"/>
+        <f t="shared" si="47"/>
         <v>1</v>
       </c>
       <c r="C101" s="9" t="s">
@@ -43654,7 +44101,10 @@
         <f>'2_CC'!I31</f>
         <v>8855442.266161751</v>
       </c>
-      <c r="I101" s="1"/>
+      <c r="I101" s="1" t="str">
+        <f t="shared" si="45"/>
+        <v>BF</v>
+      </c>
       <c r="J101" s="1">
         <f>'2_CL'!AC27</f>
         <v>1795972.3118921947</v>
@@ -43666,6 +44116,10 @@
       <c r="L101" s="5">
         <f>'2_CC'!H31</f>
         <v>3705484.266161751</v>
+      </c>
+      <c r="M101" s="1" t="str">
+        <f t="shared" si="46"/>
+        <v>BF</v>
       </c>
     </row>
     <row r="107" spans="2:27" ht="26.25" x14ac:dyDescent="0.4">
@@ -43706,79 +44160,79 @@
         <v>2</v>
       </c>
       <c r="F109" s="11">
-        <f t="shared" ref="F109:AA109" si="46">+E109+1</f>
+        <f t="shared" ref="F109:AA109" si="48">+E109+1</f>
         <v>3</v>
       </c>
       <c r="G109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>4</v>
       </c>
       <c r="H109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>5</v>
       </c>
       <c r="I109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>6</v>
       </c>
       <c r="J109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>7</v>
       </c>
       <c r="K109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>8</v>
       </c>
       <c r="L109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>9</v>
       </c>
       <c r="M109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>10</v>
       </c>
       <c r="N109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>11</v>
       </c>
       <c r="O109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>12</v>
       </c>
       <c r="P109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>13</v>
       </c>
       <c r="Q109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>14</v>
       </c>
       <c r="R109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>15</v>
       </c>
       <c r="S109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>16</v>
       </c>
       <c r="T109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>17</v>
       </c>
       <c r="U109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>18</v>
       </c>
       <c r="V109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>19</v>
       </c>
       <c r="W109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>20</v>
       </c>
       <c r="X109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>21</v>
       </c>
       <c r="Y109" s="11">
@@ -43786,11 +44240,11 @@
         <v>22</v>
       </c>
       <c r="Z109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>23</v>
       </c>
       <c r="AA109" s="11">
-        <f t="shared" si="46"/>
+        <f t="shared" si="48"/>
         <v>24</v>
       </c>
     </row>
@@ -45942,70 +46396,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="155" t="s">
+      <c r="A1" s="147" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="155"/>
-      <c r="C1" s="155"/>
-      <c r="D1" s="155"/>
-      <c r="E1" s="155"/>
-      <c r="F1" s="155"/>
-      <c r="G1" s="155"/>
-      <c r="H1" s="155"/>
-      <c r="I1" s="155"/>
-      <c r="J1" s="155"/>
-      <c r="K1" s="155"/>
-      <c r="L1" s="155"/>
-      <c r="M1" s="155"/>
-      <c r="N1" s="155"/>
-      <c r="O1" s="155"/>
-      <c r="P1" s="155"/>
-      <c r="Q1" s="155"/>
-      <c r="R1" s="155"/>
-      <c r="S1" s="155"/>
-      <c r="T1" s="155"/>
-      <c r="U1" s="155"/>
-      <c r="V1" s="155"/>
-      <c r="W1" s="155"/>
-      <c r="X1" s="155"/>
-      <c r="Y1" s="155"/>
-      <c r="Z1" s="155"/>
-      <c r="AA1" s="155"/>
-      <c r="AB1" s="155"/>
-      <c r="AC1" s="155"/>
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+      <c r="D1" s="147"/>
+      <c r="E1" s="147"/>
+      <c r="F1" s="147"/>
+      <c r="G1" s="147"/>
+      <c r="H1" s="147"/>
+      <c r="I1" s="147"/>
+      <c r="J1" s="147"/>
+      <c r="K1" s="147"/>
+      <c r="L1" s="147"/>
+      <c r="M1" s="147"/>
+      <c r="N1" s="147"/>
+      <c r="O1" s="147"/>
+      <c r="P1" s="147"/>
+      <c r="Q1" s="147"/>
+      <c r="R1" s="147"/>
+      <c r="S1" s="147"/>
+      <c r="T1" s="147"/>
+      <c r="U1" s="147"/>
+      <c r="V1" s="147"/>
+      <c r="W1" s="147"/>
+      <c r="X1" s="147"/>
+      <c r="Y1" s="147"/>
+      <c r="Z1" s="147"/>
+      <c r="AA1" s="147"/>
+      <c r="AB1" s="147"/>
+      <c r="AC1" s="147"/>
     </row>
     <row r="2" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="156" t="s">
+      <c r="A2" s="148" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="156"/>
-      <c r="C2" s="156"/>
-      <c r="D2" s="156"/>
-      <c r="E2" s="156"/>
-      <c r="F2" s="156"/>
-      <c r="G2" s="156"/>
-      <c r="H2" s="156"/>
-      <c r="I2" s="156"/>
-      <c r="J2" s="156"/>
-      <c r="K2" s="156"/>
-      <c r="L2" s="156"/>
-      <c r="M2" s="156"/>
-      <c r="N2" s="156"/>
-      <c r="O2" s="156"/>
-      <c r="P2" s="156"/>
-      <c r="Q2" s="156"/>
-      <c r="R2" s="156"/>
-      <c r="S2" s="156"/>
-      <c r="T2" s="156"/>
-      <c r="U2" s="156"/>
-      <c r="V2" s="156"/>
-      <c r="W2" s="156"/>
-      <c r="X2" s="156"/>
-      <c r="Y2" s="156"/>
-      <c r="Z2" s="156"/>
-      <c r="AA2" s="156"/>
-      <c r="AB2" s="156"/>
-      <c r="AC2" s="156"/>
+      <c r="B2" s="148"/>
+      <c r="C2" s="148"/>
+      <c r="D2" s="148"/>
+      <c r="E2" s="148"/>
+      <c r="F2" s="148"/>
+      <c r="G2" s="148"/>
+      <c r="H2" s="148"/>
+      <c r="I2" s="148"/>
+      <c r="J2" s="148"/>
+      <c r="K2" s="148"/>
+      <c r="L2" s="148"/>
+      <c r="M2" s="148"/>
+      <c r="N2" s="148"/>
+      <c r="O2" s="148"/>
+      <c r="P2" s="148"/>
+      <c r="Q2" s="148"/>
+      <c r="R2" s="148"/>
+      <c r="S2" s="148"/>
+      <c r="T2" s="148"/>
+      <c r="U2" s="148"/>
+      <c r="V2" s="148"/>
+      <c r="W2" s="148"/>
+      <c r="X2" s="148"/>
+      <c r="Y2" s="148"/>
+      <c r="Z2" s="148"/>
+      <c r="AA2" s="148"/>
+      <c r="AB2" s="148"/>
+      <c r="AC2" s="148"/>
     </row>
     <row r="3" spans="1:29" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="29" t="s">
@@ -49189,10 +49643,10 @@
       <c r="AC30" s="38"/>
     </row>
     <row r="31" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="157" t="s">
+      <c r="A31" s="149" t="s">
         <v>151</v>
       </c>
-      <c r="B31" s="157"/>
+      <c r="B31" s="149"/>
       <c r="C31" s="81">
         <f>+C30*D31</f>
         <v>1.3487353318011903</v>
@@ -49293,10 +49747,10 @@
       <c r="AC31" s="38"/>
     </row>
     <row r="32" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="157" t="s">
+      <c r="A32" s="149" t="s">
         <v>152</v>
       </c>
-      <c r="B32" s="157"/>
+      <c r="B32" s="149"/>
       <c r="C32" s="64">
         <f>1/C31</f>
         <v>0.74143531085860548</v>
@@ -49397,34 +49851,34 @@
       <c r="AC32" s="38"/>
     </row>
     <row r="33" spans="1:29" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="158" t="s">
+      <c r="A33" s="150" t="s">
         <v>150</v>
       </c>
-      <c r="B33" s="159"/>
-      <c r="C33" s="159"/>
-      <c r="D33" s="159"/>
-      <c r="E33" s="159"/>
-      <c r="F33" s="159"/>
-      <c r="G33" s="159"/>
-      <c r="H33" s="159"/>
-      <c r="I33" s="159"/>
-      <c r="J33" s="159"/>
-      <c r="K33" s="159"/>
-      <c r="L33" s="159"/>
-      <c r="M33" s="159"/>
-      <c r="N33" s="159"/>
-      <c r="O33" s="159"/>
-      <c r="P33" s="159"/>
-      <c r="Q33" s="159"/>
-      <c r="R33" s="159"/>
-      <c r="S33" s="159"/>
-      <c r="T33" s="159"/>
-      <c r="U33" s="159"/>
-      <c r="V33" s="159"/>
-      <c r="W33" s="159"/>
-      <c r="X33" s="159"/>
-      <c r="Y33" s="159"/>
-      <c r="Z33" s="160"/>
+      <c r="B33" s="151"/>
+      <c r="C33" s="151"/>
+      <c r="D33" s="151"/>
+      <c r="E33" s="151"/>
+      <c r="F33" s="151"/>
+      <c r="G33" s="151"/>
+      <c r="H33" s="151"/>
+      <c r="I33" s="151"/>
+      <c r="J33" s="151"/>
+      <c r="K33" s="151"/>
+      <c r="L33" s="151"/>
+      <c r="M33" s="151"/>
+      <c r="N33" s="151"/>
+      <c r="O33" s="151"/>
+      <c r="P33" s="151"/>
+      <c r="Q33" s="151"/>
+      <c r="R33" s="151"/>
+      <c r="S33" s="151"/>
+      <c r="T33" s="151"/>
+      <c r="U33" s="151"/>
+      <c r="V33" s="151"/>
+      <c r="W33" s="151"/>
+      <c r="X33" s="151"/>
+      <c r="Y33" s="151"/>
+      <c r="Z33" s="152"/>
       <c r="AA33" s="45">
         <f>+SUM(AA4:AA27)</f>
         <v>177559703.55329624</v>

</xml_diff>